<commit_message>
purchse schema voucher format chnaged and tested
</commit_message>
<xml_diff>
--- a/files/Faculty_Details.xlsx
+++ b/files/Faculty_Details.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="59">
   <si>
     <t>name</t>
   </si>
@@ -123,9 +123,6 @@
     <t>dharshan.pm@sece.ac.in</t>
   </si>
   <si>
-    <t>CCE</t>
-  </si>
-  <si>
     <t xml:space="preserve"> abishek.k@sece.ac.in</t>
   </si>
   <si>
@@ -165,9 +162,6 @@
     <t>Sece008</t>
   </si>
   <si>
-    <t>hodcse@sece.ac.in</t>
-  </si>
-  <si>
     <t>HOD</t>
   </si>
   <si>
@@ -183,43 +177,31 @@
     <t>Sece007</t>
   </si>
   <si>
-    <t>hodit@sece.ac.in</t>
-  </si>
-  <si>
     <t>Mohammed Mustafa M</t>
   </si>
   <si>
     <t>Sece006</t>
   </si>
   <si>
-    <t>hodaids@sece.ac.in</t>
-  </si>
-  <si>
     <t>Professor &amp; HOD</t>
   </si>
   <si>
-    <t>SECETMA002</t>
-  </si>
-  <si>
-    <t>Dr.R.MAHESWARI</t>
-  </si>
-  <si>
-    <t>MATHS</t>
-  </si>
-  <si>
-    <t>01 Aug 2008</t>
-  </si>
-  <si>
-    <t>31 May 1982</t>
-  </si>
-  <si>
-    <t>hodmaths@sece.ac.in</t>
-  </si>
-  <si>
-    <t>9976633443</t>
-  </si>
-  <si>
-    <t>Associate Professor &amp; HOD</t>
+    <t>abishekkrishnat@gmail.com</t>
+  </si>
+  <si>
+    <t>venkateswaran.c15@gmail.com</t>
+  </si>
+  <si>
+    <t>dharshanmohan2704@gmail.com</t>
+  </si>
+  <si>
+    <t>Placement</t>
+  </si>
+  <si>
+    <t>sece009</t>
+  </si>
+  <si>
+    <t>fayazahammed.m2021ecea@sece.ac.in</t>
   </si>
 </sst>
 </file>
@@ -588,7 +570,7 @@
   <cols>
     <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.85546875" customWidth="1"/>
-    <col min="3" max="3" width="28.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="45.5703125" customWidth="1"/>
     <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -636,7 +618,7 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -677,7 +659,7 @@
         <v>19</v>
       </c>
       <c r="M2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -718,7 +700,7 @@
         <v>19</v>
       </c>
       <c r="M3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -759,7 +741,7 @@
         <v>19</v>
       </c>
       <c r="M4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -776,7 +758,7 @@
         <v>9788915620</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="F5" s="2">
         <v>37397</v>
@@ -800,24 +782,24 @@
         <v>19</v>
       </c>
       <c r="M5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
         <v>34</v>
       </c>
-      <c r="B6" t="s">
-        <v>35</v>
-      </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D6">
         <v>8098616038</v>
       </c>
       <c r="E6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F6" s="2">
         <v>37443</v>
@@ -841,30 +823,30 @@
         <v>19</v>
       </c>
       <c r="M6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
         <v>37</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="D7">
         <v>7092616038</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F7" s="2">
         <v>36288</v>
       </c>
       <c r="G7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H7" s="2">
         <v>45782</v>
@@ -882,18 +864,18 @@
         <v>19</v>
       </c>
       <c r="M7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" t="s">
         <v>44</v>
       </c>
-      <c r="B9" t="s">
-        <v>45</v>
-      </c>
       <c r="C9" s="1" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="D9">
         <v>1234567890</v>
@@ -905,16 +887,16 @@
         <v>36234</v>
       </c>
       <c r="G9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H9" s="2">
         <v>45600</v>
       </c>
       <c r="I9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K9" t="b">
         <v>1</v>
@@ -923,18 +905,18 @@
         <v>19</v>
       </c>
       <c r="M9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D10">
         <v>1243567890</v>
@@ -946,16 +928,16 @@
         <v>36234</v>
       </c>
       <c r="G10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="H10" s="2">
         <v>45600</v>
       </c>
       <c r="I10" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K10" t="b">
         <v>1</v>
@@ -964,15 +946,15 @@
         <v>19</v>
       </c>
       <c r="M10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B11" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>55</v>
@@ -981,7 +963,7 @@
         <v>1254367890</v>
       </c>
       <c r="E11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F11" s="2">
         <v>36234</v>
@@ -993,10 +975,10 @@
         <v>45600</v>
       </c>
       <c r="I11" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="K11" t="b">
         <v>1</v>
@@ -1005,39 +987,39 @@
         <v>19</v>
       </c>
       <c r="M11" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B13" t="s">
         <v>57</v>
       </c>
-      <c r="C13" t="s">
-        <v>62</v>
-      </c>
-      <c r="D13" t="s">
-        <v>63</v>
+      <c r="C13" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13">
+        <v>1213456567</v>
       </c>
       <c r="E13" t="s">
-        <v>59</v>
-      </c>
-      <c r="F13" t="s">
-        <v>61</v>
+        <v>56</v>
+      </c>
+      <c r="F13" s="2">
+        <v>36234</v>
       </c>
       <c r="G13" t="s">
-        <v>41</v>
-      </c>
-      <c r="H13" t="s">
-        <v>60</v>
+        <v>16</v>
+      </c>
+      <c r="H13" s="2">
+        <v>45600</v>
       </c>
       <c r="I13" t="s">
-        <v>64</v>
-      </c>
-      <c r="J13" t="s">
-        <v>48</v>
+        <v>52</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>46</v>
       </c>
       <c r="K13" t="b">
         <v>1</v>
@@ -1046,7 +1028,7 @@
         <v>19</v>
       </c>
       <c r="M13" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1059,8 +1041,9 @@
     <hyperlink ref="C9" r:id="rId6"/>
     <hyperlink ref="C10" r:id="rId7"/>
     <hyperlink ref="C11" r:id="rId8"/>
+    <hyperlink ref="C13" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId9"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId10"/>
 </worksheet>
 </file>
</xml_diff>